<commit_message>
Add Stroop carousel PDF for Oct 15 and sync the schedule workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8uTH5muDDwNRBTTXtXiKC
</commit_message>
<xml_diff>
--- a/linkedin/programacion-linkedin-octubre-2026.xlsx
+++ b/linkedin/programacion-linkedin-octubre-2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="136">
   <si>
     <t xml:space="preserve">Programación de LinkedIn: octubre 2026</t>
   </si>
@@ -225,13 +225,10 @@
 Juégalo y cuéntame: ¿en qué ronda te enredaste?</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Confirmar con el Colegio Divino Niño si se puede nombrar; si no, usar 'un grupo de docentes en Rionegro'. 2) Diseñar el PDF del carrusel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stroop (1935); Diamond (2013); Moffitt et al. (2011), PNAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Falta diseñar el PDF</t>
+    <t xml:space="preserve">Confirmar con el Colegio Divino Niño si se puede nombrar; si no, usar 'un grupo de docentes en Rionegro'. El PDF ya está listo: carrusel-stroop-15-oct.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stroop (1935); Diamond (2013); Moffitt et al. (2011), PNAS; Diamond y Lee (2011), Science</t>
   </si>
   <si>
     <t xml:space="preserve">Por qué "no interrumpas" es tan difícil, y el parqueadero de ideas</t>
@@ -434,13 +431,13 @@
     <t xml:space="preserve">Frase grande, centrada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Y se puede entrenar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El autocontrol en la infancia predice la salud, las finanzas y el bienestar en la adultez (Moffitt et al., 2011).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente en letra pequeña abajo.</t>
+    <t xml:space="preserve">Importa, y se puede entrenar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El autocontrol en la infancia predice la salud, las finanzas y el bienestar en la adultez (Moffitt et al., 2011). Y hay programas que han mejorado las funciones ejecutivas en niños de 4 a 12 años (Diamond y Lee, 2011).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuentes en letra pequeña abajo.</t>
   </si>
   <si>
     <t xml:space="preserve">Guarda este reto para hacerlo con tu grupo</t>
@@ -452,7 +449,7 @@
     <t xml:space="preserve">Cierre con tu foto o el logo de CCA. Sin link (el post del 15 no invita al taller).</t>
   </si>
   <si>
-    <t xml:space="preserve">PDF horizontal 4:5 o cuadrado (1080 x 1080 px por página). Se sube en LinkedIn con '+' y 'Add a document'.</t>
+    <t xml:space="preserve">Listo: linkedin/carrusel-stroop-15-oct.pdf (12 páginas cuadradas de 1080 x 1080 px). Se sube en LinkedIn con '+' y 'Add a document'.</t>
   </si>
   <si>
     <t xml:space="preserve">Acción</t>
@@ -1252,7 +1249,7 @@
         <v>56</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1269,7 +1266,7 @@
         <v>32</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>51</v>
@@ -1278,23 +1275,23 @@
         <v>35</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="J5" s="8" t="n">
         <f aca="false">LEN(I5)</f>
         <v>1220</v>
       </c>
       <c r="K5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="L5" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="M5" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="N5" s="9" t="s">
         <v>48</v>
@@ -1314,19 +1311,19 @@
         <v>32</v>
       </c>
       <c r="E6" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="J6" s="8" t="n">
         <f aca="false">LEN(I6)</f>
@@ -1339,7 +1336,7 @@
         <v>46</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="N6" s="9" t="s">
         <v>48</v>
@@ -1359,19 +1356,19 @@
         <v>32</v>
       </c>
       <c r="E7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>35</v>
       </c>
       <c r="H7" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>72</v>
       </c>
       <c r="J7" s="8" t="n">
         <f aca="false">LEN(I7)</f>
@@ -1381,10 +1378,10 @@
         <v>38</v>
       </c>
       <c r="L7" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>74</v>
       </c>
       <c r="N7" s="9" t="s">
         <v>48</v>
@@ -1404,32 +1401,32 @@
         <v>32</v>
       </c>
       <c r="E8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>76</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>35</v>
       </c>
       <c r="H8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>78</v>
       </c>
       <c r="J8" s="8" t="n">
         <f aca="false">LEN(I8)</f>
         <v>1008</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L8" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="M8" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="N8" s="9" t="s">
         <v>48</v>
@@ -1478,16 +1475,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>83</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1495,13 +1492,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>86</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1509,13 +1506,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1523,13 +1520,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1537,13 +1534,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>94</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1551,13 +1548,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1565,13 +1562,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>99</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1579,13 +1576,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1593,13 +1590,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1607,13 +1604,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1621,27 +1618,27 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1649,13 +1646,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1663,7 +1660,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1693,72 +1690,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>135</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>